<commit_message>
Modified the excel path
</commit_message>
<xml_diff>
--- a/backend/reports.xlsx
+++ b/backend/reports.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FD5"/>
+  <dimension ref="A1:FD6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2338,14 +2338,11 @@
           <t>Arella on Jones</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Gloria Woolfolk</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Gloria Woolfolk; Gloria Woolfolk; Gloria Woodfolk; Gloria Rogers</t>
@@ -2384,9 +2381,6 @@
           <t>Exact match between SSN on input and on file.</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>0</v>
       </c>
@@ -2464,20 +2458,11 @@
           <t>[{"date": "07/24/2025", "name": "DHI MORTGAGE COMPANY", "kind_of_business": "Miscellaneous"}, {"date": "07/17/2025", "name": "NAVY FCU", "kind_of_business": "Credit Union and Finance Other Than Personal Companies"}, {"date": "02/01/2025", "name": "SYNCB", "kind_of_business": "Finance or Personal"}, {"date": "12/02/2024", "name": "MOVEMENT MOR", "kind_of_business": null}, {"date": "11/25/2024", "name": "DHI MORTGAGE", "kind_of_business": null}, {"date": "11/25/2024", "name": "NAVY FCU", "kind_of_business": "Credit Union and Finance Other Than Personal Companies"}, {"date": "10/26/2024", "name": "MB FIN SVCS", "kind_of_business": "Finance or Personal"}, {"date": "10/18/2024", "name": "TRUISTAUTO", "kind_of_business": "Banks"}, {"date": "10/18/2024", "name": "TD AUTO FIN", "kind_of_business": "Finance or Personal"}, {"date": "10/18/2024", "name": "MB FIN SVCS", "kind_of_business": "Finance or Personal"}, {"date": "10/18/2024", "name": "JPMCB AUTO", "kind_of_business": "Banks"}, {"date": "10/18/2024", "name": "MERCEDES BEN", "kind_of_business": "Automotive"}, {"date": "09/16/2024", "name": "NAVY FCU", "kind_of_business": "Credit Union and Finance Other Than Personal Companies"}, {"date": "06/26/2024", "name": "SYNCB/BELK", "kind_of_business": "Travel/Entertainment"}]</t>
         </is>
       </c>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="inlineStr"/>
       <c r="AY5" t="inlineStr">
         <is>
           <t>Too many recently opened accounts</t>
@@ -2537,7 +2522,6 @@
       <c r="BO5" t="n">
         <v>2713</v>
       </c>
-      <c r="BP5" t="inlineStr"/>
       <c r="BQ5" t="n">
         <v>1</v>
       </c>
@@ -2556,23 +2540,9 @@
       <c r="BV5" t="n">
         <v>1769</v>
       </c>
-      <c r="BW5" t="inlineStr"/>
       <c r="BX5" t="n">
         <v>0</v>
       </c>
-      <c r="BY5" t="inlineStr"/>
-      <c r="BZ5" t="inlineStr"/>
-      <c r="CA5" t="inlineStr"/>
-      <c r="CB5" t="inlineStr"/>
-      <c r="CC5" t="inlineStr"/>
-      <c r="CD5" t="inlineStr"/>
-      <c r="CE5" t="inlineStr"/>
-      <c r="CF5" t="inlineStr"/>
-      <c r="CG5" t="inlineStr"/>
-      <c r="CH5" t="inlineStr"/>
-      <c r="CI5" t="inlineStr"/>
-      <c r="CJ5" t="inlineStr"/>
-      <c r="CK5" t="inlineStr"/>
       <c r="CL5" t="n">
         <v>17</v>
       </c>
@@ -2591,7 +2561,6 @@
       <c r="CQ5" t="n">
         <v>4659</v>
       </c>
-      <c r="CR5" t="inlineStr"/>
       <c r="CS5" t="n">
         <v>371534</v>
       </c>
@@ -2637,10 +2606,6 @@
       <c r="DG5" t="n">
         <v>3</v>
       </c>
-      <c r="DH5" t="inlineStr"/>
-      <c r="DI5" t="inlineStr"/>
-      <c r="DJ5" t="inlineStr"/>
-      <c r="DK5" t="inlineStr"/>
       <c r="DL5" t="n">
         <v>0</v>
       </c>
@@ -2655,45 +2620,6 @@
           <t>07/24/2025</t>
         </is>
       </c>
-      <c r="DP5" t="inlineStr"/>
-      <c r="DQ5" t="inlineStr"/>
-      <c r="DR5" t="inlineStr"/>
-      <c r="DS5" t="inlineStr"/>
-      <c r="DT5" t="inlineStr"/>
-      <c r="DU5" t="inlineStr"/>
-      <c r="DV5" t="inlineStr"/>
-      <c r="DW5" t="inlineStr"/>
-      <c r="DX5" t="inlineStr"/>
-      <c r="DY5" t="inlineStr"/>
-      <c r="DZ5" t="inlineStr"/>
-      <c r="EA5" t="inlineStr"/>
-      <c r="EB5" t="inlineStr"/>
-      <c r="EC5" t="inlineStr"/>
-      <c r="ED5" t="inlineStr"/>
-      <c r="EE5" t="inlineStr"/>
-      <c r="EF5" t="inlineStr"/>
-      <c r="EG5" t="inlineStr"/>
-      <c r="EH5" t="inlineStr"/>
-      <c r="EI5" t="inlineStr"/>
-      <c r="EJ5" t="inlineStr"/>
-      <c r="EK5" t="inlineStr"/>
-      <c r="EL5" t="inlineStr"/>
-      <c r="EM5" t="inlineStr"/>
-      <c r="EN5" t="inlineStr"/>
-      <c r="EO5" t="inlineStr"/>
-      <c r="EP5" t="inlineStr"/>
-      <c r="EQ5" t="inlineStr"/>
-      <c r="ER5" t="inlineStr"/>
-      <c r="ES5" t="inlineStr"/>
-      <c r="ET5" t="inlineStr"/>
-      <c r="EU5" t="inlineStr"/>
-      <c r="EV5" t="inlineStr"/>
-      <c r="EW5" t="inlineStr"/>
-      <c r="EX5" t="inlineStr"/>
-      <c r="EY5" t="inlineStr"/>
-      <c r="EZ5" t="inlineStr"/>
-      <c r="FA5" t="inlineStr"/>
-      <c r="FB5" t="inlineStr"/>
       <c r="FC5" t="inlineStr">
         <is>
           <t>CRER_6363_524747.pdf</t>
@@ -2702,6 +2628,370 @@
       <c r="FD5" t="inlineStr">
         <is>
           <t>06/09/2026 09:31:11 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TransUnion PDF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07/09/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>System User</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>22 North</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ismael E Urbina</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>["Ismael Euceda", "Ismael Uceda"]</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>501 Horseshoe Dr, 1204 Leander TX 78641</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>512-203-8703</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Construction Leander, TX</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Exact SSN match</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Input (Current/Previous) Address is Commercial | Last name - input does not match file | Input SSN is not likely issued prior to June 2011.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U6" t="n">
+        <v>592</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>ResidentScore 4.0</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>["Too many inquiries", "Not enough available credit", "Length of time revolving accounts have been established is too short", "Too few satisfactory accounts"]</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>{"revolving": {"count": 1, "high_credit": 0, "credit_limit": 500, "balance": 0, "past_due": 0, "payment": 0, "available": 100}, "installment": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "mortgage": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "open": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "closed_w_bal": {"count": null, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "total": {"count": 1, "high_credit": 0, "credit_limit": 500, "balance": 0, "past_due": 0, "payment": 0, "available": null}}</t>
+        </is>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>[{"creditor_name": "JPMCB CARD", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving", "account_type": "Individual account", "opened": "05/25", "verified": "06/25", "closed": null, "balance": 0, "past_due": 0, "credit_limit": 500, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": "Automated account", "notes": null, "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}]</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>[{"date": "07/08/2025", "name": "ALLY FINANCI", "kind_of_business": "Finance or Personal"}, {"date": "07/08/2025", "name": "AUSTIN TELCO", "kind_of_business": "Credit Union and Finance Other Than Personal Companies"}, {"date": "07/08/2025", "name": "FIRST HELP F", "kind_of_business": "Finance or Personal"}, {"date": "07/08/2025", "name": "TOYOTA OF NO", "kind_of_business": "Automotive"}, {"date": "05/27/2025", "name": "RUNDRCKTYOTA", "kind_of_business": "Automotive"}, {"date": "05/23/2025", "name": "COVERT CHRYS", "kind_of_business": "Automotive"}, {"date": "04/28/2025", "name": "TOYOTA OF NO", "kind_of_business": "Automotive"}, {"date": "04/12/2025", "name": "SYNCB/LOWES", "kind_of_business": "Building Materials"}]</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>Too many inquiries</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>Not enough available credit</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>Length of time revolving accounts have been established is too short</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Too few satisfactory accounts</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>500</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY6" t="inlineStr"/>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>500</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR6" t="inlineStr"/>
+      <c r="CS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>500</v>
+      </c>
+      <c r="CV6" t="inlineStr"/>
+      <c r="CW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH6" t="inlineStr"/>
+      <c r="DI6" t="inlineStr"/>
+      <c r="DJ6" t="inlineStr"/>
+      <c r="DK6" t="inlineStr"/>
+      <c r="DL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM6" t="n">
+        <v>8</v>
+      </c>
+      <c r="DN6" t="n">
+        <v>7</v>
+      </c>
+      <c r="DO6" t="inlineStr">
+        <is>
+          <t>07/08/2025</t>
+        </is>
+      </c>
+      <c r="DP6" t="inlineStr"/>
+      <c r="DQ6" t="inlineStr"/>
+      <c r="DR6" t="inlineStr"/>
+      <c r="DS6" t="inlineStr"/>
+      <c r="DT6" t="inlineStr"/>
+      <c r="DU6" t="inlineStr"/>
+      <c r="DV6" t="inlineStr"/>
+      <c r="DW6" t="inlineStr"/>
+      <c r="DX6" t="inlineStr"/>
+      <c r="DY6" t="inlineStr"/>
+      <c r="DZ6" t="inlineStr"/>
+      <c r="EA6" t="inlineStr"/>
+      <c r="EB6" t="inlineStr"/>
+      <c r="EC6" t="inlineStr"/>
+      <c r="ED6" t="inlineStr"/>
+      <c r="EE6" t="inlineStr"/>
+      <c r="EF6" t="inlineStr"/>
+      <c r="EG6" t="inlineStr"/>
+      <c r="EH6" t="inlineStr"/>
+      <c r="EI6" t="inlineStr"/>
+      <c r="EJ6" t="inlineStr"/>
+      <c r="EK6" t="inlineStr"/>
+      <c r="EL6" t="inlineStr"/>
+      <c r="EM6" t="inlineStr"/>
+      <c r="EN6" t="inlineStr"/>
+      <c r="EO6" t="inlineStr"/>
+      <c r="EP6" t="inlineStr"/>
+      <c r="EQ6" t="inlineStr"/>
+      <c r="ER6" t="inlineStr"/>
+      <c r="ES6" t="inlineStr"/>
+      <c r="ET6" t="inlineStr"/>
+      <c r="EU6" t="inlineStr"/>
+      <c r="EV6" t="inlineStr"/>
+      <c r="EW6" t="inlineStr"/>
+      <c r="EX6" t="inlineStr"/>
+      <c r="EY6" t="inlineStr"/>
+      <c r="EZ6" t="inlineStr"/>
+      <c r="FA6" t="inlineStr"/>
+      <c r="FB6" t="inlineStr"/>
+      <c r="FC6" t="inlineStr">
+        <is>
+          <t>CRER_2610_517309.pdf</t>
+        </is>
+      </c>
+      <c r="FD6" t="inlineStr">
+        <is>
+          <t>06/09/2026 10:50:45 PM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Asyncio and semaphore
</commit_message>
<xml_diff>
--- a/backend/reports.xlsx
+++ b/backend/reports.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FD6"/>
+  <dimension ref="A1:FD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2652,14 +2652,11 @@
           <t>22 North</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Ismael E Urbina</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>["Ismael Euceda", "Ismael Uceda"]</t>
@@ -2673,8 +2670,6 @@
           <t>501 Horseshoe Dr, 1204 Leander TX 78641</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>512-203-8703</t>
@@ -2695,7 +2690,6 @@
           <t>Input (Current/Previous) Address is Commercial | Last name - input does not match file | Input SSN is not likely issued prior to June 2011.</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="b">
         <v>0</v>
       </c>
@@ -2776,20 +2770,11 @@
           <t>[{"date": "07/08/2025", "name": "ALLY FINANCI", "kind_of_business": "Finance or Personal"}, {"date": "07/08/2025", "name": "AUSTIN TELCO", "kind_of_business": "Credit Union and Finance Other Than Personal Companies"}, {"date": "07/08/2025", "name": "FIRST HELP F", "kind_of_business": "Finance or Personal"}, {"date": "07/08/2025", "name": "TOYOTA OF NO", "kind_of_business": "Automotive"}, {"date": "05/27/2025", "name": "RUNDRCKTYOTA", "kind_of_business": "Automotive"}, {"date": "05/23/2025", "name": "COVERT CHRYS", "kind_of_business": "Automotive"}, {"date": "04/28/2025", "name": "TOYOTA OF NO", "kind_of_business": "Automotive"}, {"date": "04/12/2025", "name": "SYNCB/LOWES", "kind_of_business": "Building Materials"}]</t>
         </is>
       </c>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
       <c r="AY6" t="inlineStr">
         <is>
           <t>Too many inquiries</t>
@@ -2834,37 +2819,12 @@
       <c r="BJ6" t="n">
         <v>0</v>
       </c>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
-      <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
       <c r="BQ6" t="n">
         <v>0</v>
       </c>
-      <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="inlineStr"/>
-      <c r="BT6" t="inlineStr"/>
-      <c r="BU6" t="inlineStr"/>
-      <c r="BV6" t="inlineStr"/>
-      <c r="BW6" t="inlineStr"/>
       <c r="BX6" t="n">
         <v>0</v>
       </c>
-      <c r="BY6" t="inlineStr"/>
-      <c r="BZ6" t="inlineStr"/>
-      <c r="CA6" t="inlineStr"/>
-      <c r="CB6" t="inlineStr"/>
-      <c r="CC6" t="inlineStr"/>
-      <c r="CD6" t="inlineStr"/>
-      <c r="CE6" t="inlineStr"/>
-      <c r="CF6" t="inlineStr"/>
-      <c r="CG6" t="inlineStr"/>
-      <c r="CH6" t="inlineStr"/>
-      <c r="CI6" t="inlineStr"/>
-      <c r="CJ6" t="inlineStr"/>
-      <c r="CK6" t="inlineStr"/>
       <c r="CL6" t="n">
         <v>1</v>
       </c>
@@ -2883,7 +2843,6 @@
       <c r="CQ6" t="n">
         <v>0</v>
       </c>
-      <c r="CR6" t="inlineStr"/>
       <c r="CS6" t="n">
         <v>0</v>
       </c>
@@ -2893,7 +2852,6 @@
       <c r="CU6" t="n">
         <v>500</v>
       </c>
-      <c r="CV6" t="inlineStr"/>
       <c r="CW6" t="n">
         <v>0</v>
       </c>
@@ -2927,10 +2885,6 @@
       <c r="DG6" t="n">
         <v>0</v>
       </c>
-      <c r="DH6" t="inlineStr"/>
-      <c r="DI6" t="inlineStr"/>
-      <c r="DJ6" t="inlineStr"/>
-      <c r="DK6" t="inlineStr"/>
       <c r="DL6" t="n">
         <v>0</v>
       </c>
@@ -2945,45 +2899,6 @@
           <t>07/08/2025</t>
         </is>
       </c>
-      <c r="DP6" t="inlineStr"/>
-      <c r="DQ6" t="inlineStr"/>
-      <c r="DR6" t="inlineStr"/>
-      <c r="DS6" t="inlineStr"/>
-      <c r="DT6" t="inlineStr"/>
-      <c r="DU6" t="inlineStr"/>
-      <c r="DV6" t="inlineStr"/>
-      <c r="DW6" t="inlineStr"/>
-      <c r="DX6" t="inlineStr"/>
-      <c r="DY6" t="inlineStr"/>
-      <c r="DZ6" t="inlineStr"/>
-      <c r="EA6" t="inlineStr"/>
-      <c r="EB6" t="inlineStr"/>
-      <c r="EC6" t="inlineStr"/>
-      <c r="ED6" t="inlineStr"/>
-      <c r="EE6" t="inlineStr"/>
-      <c r="EF6" t="inlineStr"/>
-      <c r="EG6" t="inlineStr"/>
-      <c r="EH6" t="inlineStr"/>
-      <c r="EI6" t="inlineStr"/>
-      <c r="EJ6" t="inlineStr"/>
-      <c r="EK6" t="inlineStr"/>
-      <c r="EL6" t="inlineStr"/>
-      <c r="EM6" t="inlineStr"/>
-      <c r="EN6" t="inlineStr"/>
-      <c r="EO6" t="inlineStr"/>
-      <c r="EP6" t="inlineStr"/>
-      <c r="EQ6" t="inlineStr"/>
-      <c r="ER6" t="inlineStr"/>
-      <c r="ES6" t="inlineStr"/>
-      <c r="ET6" t="inlineStr"/>
-      <c r="EU6" t="inlineStr"/>
-      <c r="EV6" t="inlineStr"/>
-      <c r="EW6" t="inlineStr"/>
-      <c r="EX6" t="inlineStr"/>
-      <c r="EY6" t="inlineStr"/>
-      <c r="EZ6" t="inlineStr"/>
-      <c r="FA6" t="inlineStr"/>
-      <c r="FB6" t="inlineStr"/>
       <c r="FC6" t="inlineStr">
         <is>
           <t>CRER_2610_517309.pdf</t>
@@ -2992,6 +2907,1959 @@
       <c r="FD6" t="inlineStr">
         <is>
           <t>06/09/2026 10:50:45 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12/28/2023</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ROSI ISELA LOPEZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Avenues At Creekside</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>31901655</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>REUBEN GARZA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>12/05/XXXX</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>641-07-XXXX</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>REUBEN GARZA | RUEBEN GARZA | RUBEN GARZA | DAVID GARZA | GARZA DAVID</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>328 AUTUMN ROUGE NEW BRAUNFELS TX 78130</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>553 CREEKSIDE CIR NEW BRAUNFELS TX 78130</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>32610 GROVE PARK DR WALLER TX 77484</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>832-625-2742</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>WARNING  -  ** The address submitted is different from those in the credit file.** | Experian (01) Inquiry/On-file current address conflict.</t>
+        </is>
+      </c>
+      <c r="S7" t="b">
+        <v>1</v>
+      </c>
+      <c r="T7" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" t="n">
+        <v>577</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>["12: The date that you opened your oldest account is too recent", "44: Too many bankcard or revolving accounts with delinquent/derogatory status", "04: The balances on your accounts are too high compared to loan amounts", "83: Lack of sufficient relevant installment account information"]</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Approved with Conditions</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>Unit Override: 486, Applicant must pay an additional deposit equal to $200.</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 550", "result": "P"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 40 % of Applicant's income.", "result": "P"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "--"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU7" t="n">
+        <v>1425</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>3562</v>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>12: The date that you opened your oldest account is too recent</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>44: Too many bankcard or revolving accounts with delinquent/derogatory status</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>04: The balances on your accounts are too high compared to loan amounts</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>83: Lack of sufficient relevant installment account information</t>
+        </is>
+      </c>
+      <c r="CY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DX7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FC7" t="inlineStr">
+        <is>
+          <t>31901655.htm</t>
+        </is>
+      </c>
+      <c r="FD7" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:27:49 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>12/15/2023 10:45:09 AM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RYAN WLODARCZYK</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Avenues At Creekside</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>31887339</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>KIMBERLY B TRAWICK</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>06/23/XXXX</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>630-72-XXXX</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>["KIMBERLY TRAWICK", "KIM TRAWICK"]</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2430 HORNED, NEW BRAUNFELS, TX 78140</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1033 NORWAY DR, SEGUIN, TX 78155</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>402 CREEKSIDE CURV, NEW BRAUNFELS, TX 78130</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>832-625-2742</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Error in SSN</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>The address submitted is different from those in the credit file. | Experian (01) Inquiry/On-file current address conflict.</t>
+        </is>
+      </c>
+      <c r="S8" t="b">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" t="n">
+        <v>464</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>["21: No open accounts in your credit file", "12: The date that you opened your oldest account is too recent", "76: You have insufficient credit history on installment loans", "05: Too many of the delinquencies on your accounts are recent"]</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>Approved with Conditions</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Applicant must pay an additional deposit</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 550", "result": "F"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 40 % of Applicant's income.", "result": "P"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "--"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU8" t="n">
+        <v>1226</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>3992</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>30.71</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>3065</v>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>21: No open accounts in your credit file</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>12: The date that you opened your oldest account is too recent</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>76: You have insufficient credit history on installment loans</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>05: Too many of the delinquencies on your accounts are recent</t>
+        </is>
+      </c>
+      <c r="CY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DX8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FC8" t="inlineStr">
+        <is>
+          <t>31887339.htm</t>
+        </is>
+      </c>
+      <c r="FD8" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:27:49 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12/8/2024 4:04:00 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ADARA COMMUNITIES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Avenues At Creekside</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>32408294</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CATHERINE HARPEER</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>05/13/XXXX</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>462-11-XXXX</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>["CATHERINE HARPER", "KATHY HARPER", "CATHY L HARPER", "KATHERINE HARPER"]</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>LIVING WITH, SAN MARCOS, TX 78666</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1615 REDWOOD RD APT 26D SAN MARCOS TX 78666</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1320 WILSON ST APT 230 LOCKHART TX 78644</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>832-625-2742</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>WARNING  -  ** The address submitted is different from those in the credit file.** | Experian (01) Inquiry/On-file current address conflict.</t>
+        </is>
+      </c>
+      <c r="S9" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" t="n">
+        <v>2</v>
+      </c>
+      <c r="U9" t="n">
+        <v>510</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>["04: The balances on your accounts are too high compared to loan amounts", "12: The date that you opened your oldest account is too recent", "61: No open real estate accounts in your credit file", "95: You have too many collection agency accounts that are unpaid"]</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>Rejected: Applicant failed criteria 132 which has no override.</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 550", "result": "F"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 40 % of Applicant's income.", "result": "P"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "--"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>4500</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>2498</v>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>04: The balances on your accounts are too high compared to loan amounts</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>12: The date that you opened your oldest account is too recent</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>61: No open real estate accounts in your credit file</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>95: You have too many collection agency accounts that are unpaid</t>
+        </is>
+      </c>
+      <c r="CY9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DX9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FC9" t="inlineStr">
+        <is>
+          <t>32408294.htm</t>
+        </is>
+      </c>
+      <c r="FD9" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:27:51 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4/21/2025</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SIBONNE ALEXIS MURPH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Avenues At Creekside</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>32567346</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ROGER O HERRERA LOPEZ</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>04/15/XXXX</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>633-23-XXXX</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>["ROGER HERRERALOPEZ"]</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2534 MCCRAE, NEW BRAUNFELS, TX 78130</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>832-625-2742</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>WARNING  -  ** The address submitted is different from those in the credit file.** | Experian (01) Inquiry/On-file current address conflict.</t>
+        </is>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="n">
+        <v>2</v>
+      </c>
+      <c r="U10" t="n">
+        <v>746</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>["43: Lack of sufficient credit history on bankcard or revolving accounts", "85: You have too many inquiries on your credit report", "08: You have either too few loans or too many loans with recent delinquencies", "65: Lack of sufficient relevant first mortgage account information"]</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "P"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 550", "result": "P"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 40 % of Applicant's income.", "result": "--"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "P"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AV10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>43: Lack of sufficient credit history on bankcard or revolving accounts</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>85: You have too many inquiries on your credit report</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>08: You have either too few loans or too many loans with recent delinquencies</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>65: Lack of sufficient relevant first mortgage account information</t>
+        </is>
+      </c>
+      <c r="CY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DW10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DX10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="FC10" t="inlineStr">
+        <is>
+          <t>32567346.htm</t>
+        </is>
+      </c>
+      <c r="FD10" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:27:51 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TransUnion PDF</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>8/8/2025</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>System User</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Avenues at Creekside</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cheryl L Fann</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Cheryl Fann; Cheryl Smith</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>770 N Interstate 35, 214 New Braunfels TX 78130</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>7635 Bandera Rd, 12208 San Antonio TX 78238</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>4801 Gus Eckert Rd, 308 San Antonio TX 78240</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>210-984-4156</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Heb
+San Antonio, TX
+Valeroarant Agency</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Exact SSN match</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Current address mismatch - Input does not match file.</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1</v>
+      </c>
+      <c r="U11" t="n">
+        <v>729</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>ResidentScore 4.0</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>["Too many different phone numbers reported", "Length at current reported residence is too short", "Balance of non-mortgage accounts is too high", "Not enough available credit on active or open bankcard accounts"]</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>35</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>{"revolving": {"count": 7, "high_credit": 13666, "credit_limit": 15550, "balance": 9379, "past_due": 0, "payment": 274, "available": "40%"}, "installment": {"count": 28, "high_credit": 61495, "credit_limit": 0, "balance": 69456, "past_due": 0, "payment": 562, "available": null}, "mortgage": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "open": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "closed_w_bal": {"count": null, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "total": {"count": 35, "high_credit": 75161, "credit_limit": 15550, "balance": 78835, "past_due": 0, "payment": 836, "available": null}}</t>
+        </is>
+      </c>
+      <c r="AH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>[{"creditor_name": "SYNCB/CC DC", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving MIN", "account_type": "Individual account", "opened": null, "verified": null, "closed": null, "balance": null, "past_due": null, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "THD/CBNA", "industry": "Banks", "loan_type": "Charge Account", "loan_terms": "Revolving", "account_type": null, "opened": "01/25", "verified": "07/25", "closed": null, "balance": 0, "past_due": 0, "credit_limit": 4000, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "CAPITAL ONE", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving", "account_type": "Individual account", "opened": "09/23", "verified": "07/25", "closed": null, "balance": 0, "past_due": 0, "credit_limit": 500, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "UPSTA/FINWSE", "industry": "Finance or Personal", "loan_type": "Unsecured", "loan_terms": null, "account_type": "Individual account", "opened": "11/24", "verified": "07/25", "closed": null, "balance": 7052, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": null, "industry": null, "loan_type": null, "loan_terms": null, "account_type": null, "opened": "06/22", "verified": "08/25", "closed": null, "balance": 1211, "past_due": 0, "credit_limit": 1300, "payment_amount": 40, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": null, "industry": null, "loan_type": "Installment", "loan_terms": "060 Monthly", "account_type": "Individual account", "opened": null, "verified": null, "closed": null, "balance": 15550, "past_due": 0, "credit_limit": null, "payment_amount": 241, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "IMPRINTPAYM", "industry": "Finance or Personal", "loan_type": null, "loan_terms": null, "account_type": null, "opened": "01/25", "verified": "07/25", "closed": null, "balance": 1780, "past_due": 0, "credit_limit": 2000, "payment_amount": 58, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "CAPITAL ONE", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving MIN", "account_type": "Individual account", "opened": "07/21", "verified": "07/25", "closed": null, "balance": null, "past_due": null, "credit_limit": 1250, "payment_amount": 28, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "CAPITAL ONE", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving MIN", "account_type": "Individual account", "opened": "09/18", "verified": "07/25", "closed": null, "balance": 3445, "past_due": 0, "credit_limit": 3500, "payment_amount": 108, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": null, "industry": null, "loan_type": "Credit Card", "loan_terms": "Revolving MIN", "account_type": "Individual account", "opened": null, "verified": null, "closed": null, "balance": 243, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "JPMCB CARD", "industry": "Banks", "loan_type": "Flexible Spending Credit Card", "loan_terms": "Revolving MIN", "account_type": "Individual account", "opened": "10/24", "verified": "07/25", "closed": null, "balance": 2700, "past_due": 0, "credit_limit": 3000, "payment_amount": 40, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "UPSTART NETW", "industry": "Finance or Personal", "loan_type": "Unsecured", "loan_terms": "Installment 018 Monthly", "account_type": "Individual account", "opened": "06/25", "verified": "07/25", "closed": null, "balance": 2955, "past_due": 0, "credit_limit": null, "payment_amount": 173, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}]</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>[{"date": "06/05/2025", "name": "CRB/UPSTART", "kind_of_business": "Finance or Personal"}, {"date": "01/17/2025", "name": "FEB/IMPRINT", "kind_of_business": "Finance or Personal"}, {"date": "11/21/2024", "name": "FINWISE/UPST", "kind_of_business": "Finance or Personal"}, {"date": "01/24/2024", "name": "JPMCB CARD", "kind_of_business": "Banks"}, {"date": "12/19/2023", "name": "SYNCB/AMAZON", "kind_of_business": "Banks"}, {"date": "11/14/2023", "name": "1ST FRANKLIN", "kind_of_business": "Finance or Personal"}, {"date": "09/28/2023", "name": "CAPITAL ONE", "kind_of_business": "Banks"}]</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>Too many different phone numbers reported</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>Length at current reported residence is too short</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>Balance of non-mortgage accounts is too high</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>Not enough available credit on active or open bankcard accounts</t>
+        </is>
+      </c>
+      <c r="BC11" t="n">
+        <v>7</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>13666</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>15550</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>9379</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>274</v>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="BJ11" t="n">
+        <v>28</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>61495</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>69456</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>562</v>
+      </c>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
+      <c r="BX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY11" t="inlineStr"/>
+      <c r="BZ11" t="inlineStr"/>
+      <c r="CA11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr"/>
+      <c r="CC11" t="inlineStr"/>
+      <c r="CD11" t="inlineStr"/>
+      <c r="CE11" t="inlineStr"/>
+      <c r="CF11" t="inlineStr"/>
+      <c r="CG11" t="inlineStr"/>
+      <c r="CH11" t="inlineStr"/>
+      <c r="CI11" t="inlineStr"/>
+      <c r="CJ11" t="inlineStr"/>
+      <c r="CK11" t="inlineStr"/>
+      <c r="CL11" t="n">
+        <v>35</v>
+      </c>
+      <c r="CM11" t="n">
+        <v>75161</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>15550</v>
+      </c>
+      <c r="CO11" t="n">
+        <v>78835</v>
+      </c>
+      <c r="CP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ11" t="n">
+        <v>836</v>
+      </c>
+      <c r="CR11" t="inlineStr"/>
+      <c r="CS11" t="n">
+        <v>34936</v>
+      </c>
+      <c r="CT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU11" t="n">
+        <v>15550</v>
+      </c>
+      <c r="CV11" t="n">
+        <v>688</v>
+      </c>
+      <c r="CW11" t="n">
+        <v>15550</v>
+      </c>
+      <c r="CX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB11" t="n">
+        <v>12</v>
+      </c>
+      <c r="DC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH11" t="inlineStr"/>
+      <c r="DI11" t="inlineStr"/>
+      <c r="DJ11" t="inlineStr"/>
+      <c r="DK11" t="inlineStr"/>
+      <c r="DL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM11" t="n">
+        <v>7</v>
+      </c>
+      <c r="DN11" t="n">
+        <v>7</v>
+      </c>
+      <c r="DO11" t="inlineStr">
+        <is>
+          <t>06/05/2025</t>
+        </is>
+      </c>
+      <c r="DP11" t="inlineStr"/>
+      <c r="DQ11" t="inlineStr"/>
+      <c r="DR11" t="inlineStr"/>
+      <c r="DS11" t="inlineStr"/>
+      <c r="DT11" t="inlineStr"/>
+      <c r="DU11" t="inlineStr"/>
+      <c r="DV11" t="inlineStr"/>
+      <c r="DW11" t="inlineStr"/>
+      <c r="DX11" t="inlineStr"/>
+      <c r="DY11" t="inlineStr"/>
+      <c r="DZ11" t="inlineStr"/>
+      <c r="EA11" t="inlineStr"/>
+      <c r="EB11" t="inlineStr"/>
+      <c r="EC11" t="inlineStr"/>
+      <c r="ED11" t="inlineStr"/>
+      <c r="EE11" t="inlineStr"/>
+      <c r="EF11" t="inlineStr"/>
+      <c r="EG11" t="inlineStr"/>
+      <c r="EH11" t="inlineStr"/>
+      <c r="EI11" t="inlineStr"/>
+      <c r="EJ11" t="inlineStr"/>
+      <c r="EK11" t="inlineStr"/>
+      <c r="EL11" t="inlineStr"/>
+      <c r="EM11" t="inlineStr"/>
+      <c r="EN11" t="inlineStr"/>
+      <c r="EO11" t="inlineStr"/>
+      <c r="EP11" t="inlineStr"/>
+      <c r="EQ11" t="inlineStr"/>
+      <c r="ER11" t="inlineStr"/>
+      <c r="ES11" t="inlineStr"/>
+      <c r="ET11" t="inlineStr"/>
+      <c r="EU11" t="inlineStr"/>
+      <c r="EV11" t="inlineStr"/>
+      <c r="EW11" t="inlineStr"/>
+      <c r="EX11" t="inlineStr"/>
+      <c r="EY11" t="inlineStr"/>
+      <c r="EZ11" t="inlineStr"/>
+      <c r="FA11" t="inlineStr"/>
+      <c r="FB11" t="inlineStr"/>
+      <c r="FC11" t="inlineStr">
+        <is>
+          <t>CRER_4129_520508.pdf</t>
+        </is>
+      </c>
+      <c r="FD11" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:30:29 PM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Azure Deployment Files
</commit_message>
<xml_diff>
--- a/backend/reports.xlsx
+++ b/backend/reports.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FD11"/>
+  <dimension ref="A1:FD21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4496,14 +4496,11 @@
           <t>Avenues at Creekside</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>Cheryl L Fann</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Cheryl Fann; Cheryl Smith</t>
@@ -4549,7 +4546,6 @@
           <t>Current address mismatch - Input does not match file.</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="b">
         <v>1</v>
       </c>
@@ -4630,20 +4626,11 @@
           <t>[{"date": "06/05/2025", "name": "CRB/UPSTART", "kind_of_business": "Finance or Personal"}, {"date": "01/17/2025", "name": "FEB/IMPRINT", "kind_of_business": "Finance or Personal"}, {"date": "11/21/2024", "name": "FINWISE/UPST", "kind_of_business": "Finance or Personal"}, {"date": "01/24/2024", "name": "JPMCB CARD", "kind_of_business": "Banks"}, {"date": "12/19/2023", "name": "SYNCB/AMAZON", "kind_of_business": "Banks"}, {"date": "11/14/2023", "name": "1ST FRANKLIN", "kind_of_business": "Finance or Personal"}, {"date": "09/28/2023", "name": "CAPITAL ONE", "kind_of_business": "Banks"}]</t>
         </is>
       </c>
-      <c r="AO11" t="inlineStr"/>
-      <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AR11" t="inlineStr"/>
-      <c r="AS11" t="inlineStr"/>
-      <c r="AT11" t="inlineStr"/>
-      <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr"/>
-      <c r="AX11" t="inlineStr"/>
       <c r="AY11" t="inlineStr">
         <is>
           <t>Too many different phone numbers reported</t>
@@ -4705,32 +4692,12 @@
       <c r="BO11" t="n">
         <v>562</v>
       </c>
-      <c r="BP11" t="inlineStr"/>
       <c r="BQ11" t="n">
         <v>0</v>
       </c>
-      <c r="BR11" t="inlineStr"/>
-      <c r="BS11" t="inlineStr"/>
-      <c r="BT11" t="inlineStr"/>
-      <c r="BU11" t="inlineStr"/>
-      <c r="BV11" t="inlineStr"/>
-      <c r="BW11" t="inlineStr"/>
       <c r="BX11" t="n">
         <v>0</v>
       </c>
-      <c r="BY11" t="inlineStr"/>
-      <c r="BZ11" t="inlineStr"/>
-      <c r="CA11" t="inlineStr"/>
-      <c r="CB11" t="inlineStr"/>
-      <c r="CC11" t="inlineStr"/>
-      <c r="CD11" t="inlineStr"/>
-      <c r="CE11" t="inlineStr"/>
-      <c r="CF11" t="inlineStr"/>
-      <c r="CG11" t="inlineStr"/>
-      <c r="CH11" t="inlineStr"/>
-      <c r="CI11" t="inlineStr"/>
-      <c r="CJ11" t="inlineStr"/>
-      <c r="CK11" t="inlineStr"/>
       <c r="CL11" t="n">
         <v>35</v>
       </c>
@@ -4749,7 +4716,6 @@
       <c r="CQ11" t="n">
         <v>836</v>
       </c>
-      <c r="CR11" t="inlineStr"/>
       <c r="CS11" t="n">
         <v>34936</v>
       </c>
@@ -4795,10 +4761,6 @@
       <c r="DG11" t="n">
         <v>0</v>
       </c>
-      <c r="DH11" t="inlineStr"/>
-      <c r="DI11" t="inlineStr"/>
-      <c r="DJ11" t="inlineStr"/>
-      <c r="DK11" t="inlineStr"/>
       <c r="DL11" t="n">
         <v>0</v>
       </c>
@@ -4813,45 +4775,6 @@
           <t>06/05/2025</t>
         </is>
       </c>
-      <c r="DP11" t="inlineStr"/>
-      <c r="DQ11" t="inlineStr"/>
-      <c r="DR11" t="inlineStr"/>
-      <c r="DS11" t="inlineStr"/>
-      <c r="DT11" t="inlineStr"/>
-      <c r="DU11" t="inlineStr"/>
-      <c r="DV11" t="inlineStr"/>
-      <c r="DW11" t="inlineStr"/>
-      <c r="DX11" t="inlineStr"/>
-      <c r="DY11" t="inlineStr"/>
-      <c r="DZ11" t="inlineStr"/>
-      <c r="EA11" t="inlineStr"/>
-      <c r="EB11" t="inlineStr"/>
-      <c r="EC11" t="inlineStr"/>
-      <c r="ED11" t="inlineStr"/>
-      <c r="EE11" t="inlineStr"/>
-      <c r="EF11" t="inlineStr"/>
-      <c r="EG11" t="inlineStr"/>
-      <c r="EH11" t="inlineStr"/>
-      <c r="EI11" t="inlineStr"/>
-      <c r="EJ11" t="inlineStr"/>
-      <c r="EK11" t="inlineStr"/>
-      <c r="EL11" t="inlineStr"/>
-      <c r="EM11" t="inlineStr"/>
-      <c r="EN11" t="inlineStr"/>
-      <c r="EO11" t="inlineStr"/>
-      <c r="EP11" t="inlineStr"/>
-      <c r="EQ11" t="inlineStr"/>
-      <c r="ER11" t="inlineStr"/>
-      <c r="ES11" t="inlineStr"/>
-      <c r="ET11" t="inlineStr"/>
-      <c r="EU11" t="inlineStr"/>
-      <c r="EV11" t="inlineStr"/>
-      <c r="EW11" t="inlineStr"/>
-      <c r="EX11" t="inlineStr"/>
-      <c r="EY11" t="inlineStr"/>
-      <c r="EZ11" t="inlineStr"/>
-      <c r="FA11" t="inlineStr"/>
-      <c r="FB11" t="inlineStr"/>
       <c r="FC11" t="inlineStr">
         <is>
           <t>CRER_4129_520508.pdf</t>
@@ -4860,6 +4783,3537 @@
       <c r="FD11" t="inlineStr">
         <is>
           <t>06/10/2026 07:30:29 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2/7/2024 3:19:57 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ETHAN PAGE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>31959125</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>RICHARD CAPOZZI</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>05/31/XXXX</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>082-66-XXXX</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>["RICHARD CAPOZZI"]</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>3300 BAY SARASOTA, FL 34234</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>4715 WALDEN CIR APT 610 ORLANDO FL 32811</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2041 9TH ST SARASOTA FL 34237</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>941-351-3595</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>WARNING  -  ** The address submitted is different from those in the credit file.** | Experian (01) Inquiry/On-file current address conflict.</t>
+        </is>
+      </c>
+      <c r="S12" t="b">
+        <v>1</v>
+      </c>
+      <c r="T12" t="n">
+        <v>2</v>
+      </c>
+      <c r="U12" t="n">
+        <v>531</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>["97: You have too few credit accounts", "08: You have either too few loans or too many loans with recent delinquencies", "15: Newest delinquent/derogatory payment status on your accts is too recent", "34: Total of all balances on bankcard or revolving accounts is too high"]</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>Approved with Conditions</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Unit Override: 486, Applicant must pay an additional deposit equal to $200.</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 525", "result": "P"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 36 % of Applicant's income.", "result": "--"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "--"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU12" t="n">
+        <v>1665</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>2750</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>30.27</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>4625</v>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>97: You have too few credit accounts</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>08: You have either too few loans or too many loans with recent delinquencies</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>15: Newest delinquent/derogatory payment status on your accts is too recent</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>34: Total of all balances on bankcard or revolving accounts is too high</t>
+        </is>
+      </c>
+      <c r="CY12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV12" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DX12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB12" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="FC12" t="inlineStr">
+        <is>
+          <t>31959125.htm</t>
+        </is>
+      </c>
+      <c r="FD12" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:15 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TransUnion PDF</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>9/16/2025</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>System User</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Leonel Arriaza terraza</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>["Leonel Arriazaterraza", "Leonel Arriaza", "Leonel Terrazaarriazaterraza"]</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>5009 W Crystal Ln Santa Ana CA 92704</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>4926 W Division St Chicago IL 60651</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>949-244-1611</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Exact SSN match</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Current address mismatch - Input does not match file. | Input SSN is not likely issued prior to June 2011.</t>
+        </is>
+      </c>
+      <c r="S13" t="b">
+        <v>1</v>
+      </c>
+      <c r="T13" t="n">
+        <v>2</v>
+      </c>
+      <c r="U13" t="n">
+        <v>592</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>ResidentScore 4.0</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>["Not enough available credit", "Balance of non-mortgage accounts is too high", "Insufficient payment activity", "Not enough balance decreases on active non-mortgage accounts"]</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>{"revolving": {"count": 2, "high_credit": 1198, "credit_limit": 1198, "balance": 845, "past_due": 525, "payment": 89, "available": 0.29}, "installment": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "mortgage": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "open": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "closed_w_bal": {"count": null, "high_credit": null, "credit_limit": null, "balance": 464, "past_due": 464, "payment": 0, "available": null}, "total": {"count": 2, "high_credit": 1198, "credit_limit": 1198, "balance": 1309, "past_due": 989, "payment": 89, "available": null}}</t>
+        </is>
+      </c>
+      <c r="AH13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>[{"creditor_name": "BK OF AMER", "industry": "Banks", "loan_type": "Secured Credit Card", "loan_terms": "Revolving", "account_type": "Individual account", "opened": "11/22", "verified": "08/25", "closed": "09/24", "balance": 464, "past_due": 464, "credit_limit": null, "payment_amount": null, "status": "Charged off as Bad Debt", "remarks": "Account closed by credit grantor", "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "CURACAO", "industry": "Home/Office Furnishings", "loan_type": "Charge Account", "loan_terms": "Revolving MIN", "account_type": "Individual account", "opened": "08/22", "verified": "09/24", "closed": null, "balance": 845, "past_due": 525, "credit_limit": 1198, "payment_amount": 89, "status": "120 days past due", "remarks": null, "notes": "Automated account", "late_30": 2, "late_60": 2, "late_90": 2, "late_120_plus": 2}]</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>Not enough available credit</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>Balance of non-mortgage accounts is too high</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>Insufficient payment activity</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>Not enough balance decreases on active non-mortgage accounts</t>
+        </is>
+      </c>
+      <c r="BC13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>1198</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>1198</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>845</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>525</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>89</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH13" t="n">
+        <v>464</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>464</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL13" t="n">
+        <v>2</v>
+      </c>
+      <c r="CM13" t="n">
+        <v>1198</v>
+      </c>
+      <c r="CN13" t="n">
+        <v>1198</v>
+      </c>
+      <c r="CO13" t="n">
+        <v>1309</v>
+      </c>
+      <c r="CP13" t="n">
+        <v>989</v>
+      </c>
+      <c r="CQ13" t="n">
+        <v>89</v>
+      </c>
+      <c r="CS13" t="n">
+        <v>1309</v>
+      </c>
+      <c r="CT13" t="n">
+        <v>989</v>
+      </c>
+      <c r="CU13" t="n">
+        <v>1198</v>
+      </c>
+      <c r="CV13" t="n">
+        <v>89</v>
+      </c>
+      <c r="CW13" t="n">
+        <v>845</v>
+      </c>
+      <c r="CX13" t="n">
+        <v>525</v>
+      </c>
+      <c r="CY13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA13" t="n">
+        <v>2</v>
+      </c>
+      <c r="DB13" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC13" t="n">
+        <v>2</v>
+      </c>
+      <c r="DD13" t="n">
+        <v>2</v>
+      </c>
+      <c r="DE13" t="n">
+        <v>2</v>
+      </c>
+      <c r="DF13" t="n">
+        <v>2</v>
+      </c>
+      <c r="DG13" t="n">
+        <v>1</v>
+      </c>
+      <c r="DL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC13" t="inlineStr">
+        <is>
+          <t>CRER_5510_523152.pdf</t>
+        </is>
+      </c>
+      <c r="FD13" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:16 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TransUnion PDF</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10/6/2025</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>System User</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Cleiton Ferreira cunha</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>4212 Locust Av Sarasota FL 34234</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>941-271-2373</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>No SSN on input or on file.</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>SSN mismatch - input does not match file | Input SSN likely not issued prior to June 2011</t>
+        </is>
+      </c>
+      <c r="S14" t="b">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>2</v>
+      </c>
+      <c r="U14" t="n">
+        <v>604</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>ResidentScore 4.0</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>["Not enough available credit", "Balance of non-mortgage accounts is too high", "Too many different phone numbers reported", "Insufficient payment activity"]</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>{"revolving": {"count": 1, "high_credit": 1979, "credit_limit": 1900, "balance": 1730, "past_due": 0, "payment": 59, "available": 9}, "installment": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "mortgage": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "open": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "closed_w_bal": {"count": null, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "total": {"count": 1, "high_credit": 1979, "credit_limit": 1900, "balance": 1730, "past_due": 0, "payment": 59, "available": null}}</t>
+        </is>
+      </c>
+      <c r="AH14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>[{"creditor_name": "JPMCB CARD", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving MIN", "account_type": "Individual account for sole use of consumer", "opened": "03/24", "verified": "09/25", "closed": null, "balance": 1730, "past_due": 0, "credit_limit": 1900, "payment_amount": 59, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}]</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>Not enough available credit</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>Balance of non-mortgage accounts is too high</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>Too many different phone numbers reported</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>Insufficient payment activity</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>1979</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>1900</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>1730</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>59</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>9</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM14" t="n">
+        <v>1979</v>
+      </c>
+      <c r="CN14" t="n">
+        <v>1900</v>
+      </c>
+      <c r="CO14" t="n">
+        <v>1730</v>
+      </c>
+      <c r="CP14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ14" t="n">
+        <v>59</v>
+      </c>
+      <c r="CS14" t="n">
+        <v>1730</v>
+      </c>
+      <c r="CT14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU14" t="n">
+        <v>1900</v>
+      </c>
+      <c r="CV14" t="n">
+        <v>59</v>
+      </c>
+      <c r="CW14" t="n">
+        <v>1730</v>
+      </c>
+      <c r="CX14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB14" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC14" t="inlineStr">
+        <is>
+          <t>CRER_6164_524395.pdf</t>
+        </is>
+      </c>
+      <c r="FD14" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:23 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10/11/2021</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>YOTTA ADMIN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>30441103</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>JESUSNEY SILVA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4/12/XXXX</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>5707 29TH, BRADENTON, FL 34203</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>941-351-3595</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>{"revolving": null, "installment": null, "mortgage": null, "open": null, "closed_w_bal": null, "total": null}</t>
+        </is>
+      </c>
+      <c r="AH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>Approved with Conditions</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Unit Override: 505, Applicant must pay an additional deposit. Approve with $200.00 floor plan deposit plus $1255.00 credit risk fee.</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 84 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR112", "description": "Applicant has less than 100 % negative credit", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $300 of outstanding debt to previous landlords in the last 60 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 60 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 60 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 525", "result": "P"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 25 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 34 % of Applicant's income.", "result": "--"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "P"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 60 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 36 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 300 of outstanding rental collections debt in the past 60 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 60 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 36 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 60 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW853", "description": "Applicant has no Lease Violation records in the last 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU15" t="n">
+        <v>1455</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>6450</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>22.56</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>4279</v>
+      </c>
+      <c r="CY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DR15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV15" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DX15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EX15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA15" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB15" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="FC15" t="inlineStr">
+        <is>
+          <t>30441103.htm</t>
+        </is>
+      </c>
+      <c r="FD15" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:25 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3/18/2024</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MARIA ALVISO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>32023657</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>BAYARDO HIDALGO</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01/04/XXXX</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>817-74-XXXX</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>["BAYARDO HIDALGO"]</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>509 HEINEMAN, DAYTONA, FL 32114</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>941-351-3595</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Input Social Security Number issue date cannot be verified.</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>04- Input Social Security issue date cannot be verified.("The inquired SSN has not been issued or issued after June 2011.") | 0027 CKPT: INPUT SSN ISSUE DATE UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="S16" t="b">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>2</v>
+      </c>
+      <c r="U16" t="n">
+        <v>550</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>["97: You have too few credit accounts", "04: The balances on your accounts are too high compared to loan amounts", "63: Lack of sufficient relevant real estate account information", "32: Balances on bankcard/revolving accts too high compared to credit limits"]</t>
+        </is>
+      </c>
+      <c r="AC16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="AH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>Approved with Conditions</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Unit Override: 510, Applicant must pay an additional deposit equal to 1 months rent</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "P"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 525", "result": "P"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 36 % of Applicant's income.", "result": "P"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "--"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "F"}]</t>
+        </is>
+      </c>
+      <c r="AR16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU16" t="n">
+        <v>1549</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>8600</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>18.01</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>4303</v>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>97: You have too few credit accounts</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>04: The balances on your accounts are too high compared to loan amounts</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>63: Lack of sufficient relevant real estate account information</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>32: Balances on bankcard/revolving accts too high compared to credit limits</t>
+        </is>
+      </c>
+      <c r="CY16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DQ16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV16" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DX16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ16" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="FA16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB16" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FC16" t="inlineStr">
+        <is>
+          <t>32023657.htm</t>
+        </is>
+      </c>
+      <c r="FD16" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:27 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11/9/2024</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GLEIDY  FERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>32379239</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>BRENO  NOCERA</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>10/10/XXXX</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>350 N, SARASOTA, FL 34232</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>941-351-3595</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>{"revolving": null, "installment": null, "mortgage": null, "open": null, "closed_w_bal": null, "total": null}</t>
+        </is>
+      </c>
+      <c r="AH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>Applicant has no credit report to evaluate. The Credit (CR) and Residential History (RH) criteria will be set to the values assigned by the Management Company or Property. Rejected: Applicant failed criteria 132 which has no override.</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "F"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 525", "result": "F"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 36 % of Applicant's income.", "result": "--"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "P"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "F"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU17" t="n">
+        <v>1679</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>5400</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>31.09</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>4664</v>
+      </c>
+      <c r="CY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP17" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DQ17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV17" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW17" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DX17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY17" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="EZ17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB17" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="FC17" t="inlineStr">
+        <is>
+          <t>32379239.htm</t>
+        </is>
+      </c>
+      <c r="FD17" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:30 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>9/10/2024</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GLEIDY  FERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>32299420</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FABIO  BRAGAIOLLI</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>10/3/XXXX</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>351-53-XXXX</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>185    MIDWEST
+SARASOTA, FL  34232</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>941-351-3595</t>
+        </is>
+      </c>
+      <c r="S18" t="b">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>{"revolving": null, "installment": null, "mortgage": null, "open": null, "closed_w_bal": null, "total": null}</t>
+        </is>
+      </c>
+      <c r="AH18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>Applicant has no credit report to evaluate.  The Credit (CR) and Residential History (RH) criteria will be set to the values assigned by the Management Company or Property. Rejected: Applicant failed criteria 132 which has no override.</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "F"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 525", "result": "F"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 36 % of Applicant's income.", "result": "--"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "P"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "P"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "P"}]</t>
+        </is>
+      </c>
+      <c r="AR18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU18" t="n">
+        <v>1549</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>5600</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>27.66</v>
+      </c>
+      <c r="AX18" t="n">
+        <v>4303</v>
+      </c>
+      <c r="CY18" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP18" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DQ18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV18" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW18" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DX18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EZ18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FA18" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB18" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="FC18" t="inlineStr">
+        <is>
+          <t>32299420.htm</t>
+        </is>
+      </c>
+      <c r="FD18" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:32 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HTML Screening Report</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>8/17/2024</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GLEIDY  FERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Timberlake</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>32268854</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ODAIR  FERREIRA DE SOUZA</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1/14/XXXX</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>8437 GARDEN, SARASOTA, FL 34243</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>941-351-3595</t>
+        </is>
+      </c>
+      <c r="S19" t="b">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>{"revolving": null, "installment": null, "mortgage": null, "open": null, "closed_w_bal": null, "total": null}</t>
+        </is>
+      </c>
+      <c r="AH19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Applicant has no credit report to evaluate. The Credit (CR) and Residential History (RH) criteria will be set to the values assigned by the Management Company or Property. Rejected: Applicant failed criteria 132 which has no override.</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>[{"code": "CR100", "description": "Applicant has established credit history in the last 36 months.", "result": "F"}, {"code": "CR101", "description": "Applicant has no bankruptcy in the last 60 months.", "result": "P"}, {"code": "CR126", "description": "Applicant has less than $500 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR127", "description": "Applicant has less than $1501 of outstanding debt to previous landlords in the last 36 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR128", "description": "Applicant has outstanding debt to less than 2 previous landlords in the last 48 months as reported by the Credit Bureau.", "result": "P"}, {"code": "CR131", "description": "Applicants Credit Score is greater than or equal to 600", "result": "F"}, {"code": "CR132", "description": "Applicants Credit Score is greater than or equal to 525", "result": "F"}, {"code": "GS306", "description": "There are no records found on the Global Sanctions watch lists (including OFAC, OFAC SDN, OFAC Non-SDN and other sanction/terrorist watch lists).", "result": "P"}, {"code": "CM321", "description": "Applicant has no felony drug records in the last 25 years.", "result": "P"}, {"code": "CM322", "description": "Applicant has no misdemeanor drug records in the last 2 years.", "result": "P"}, {"code": "CM323", "description": "Applicant has no felony DUI records in the last 25 years.", "result": "P"}, {"code": "CM325", "description": "Applicant has no unclassified felony records in the last 25 years.", "result": "P"}, {"code": "CM326", "description": "Applicant has no unclassified misdemeanor records in the last 5 years.", "result": "P"}, {"code": "CM327", "description": "Applicant has no felony property records in the last 25 years.", "result": "P"}, {"code": "CM328", "description": "Applicant has no misdemeanor property records in the last 5 years.", "result": "P"}, {"code": "CM329", "description": "Applicant has no felony sex records in the last 100 years.", "result": "P"}, {"code": "CM330", "description": "Applicant has no misdemeanor sex records in the last 100 years.", "result": "P"}, {"code": "CM331", "description": "Applicant has no felony theft records in the last 25 years.", "result": "P"}, {"code": "CM332", "description": "Applicant has no misdemeanor theft records in the last 5 years.", "result": "P"}, {"code": "CM333", "description": "Applicant has no felony theft by check records in the last 25 years.", "result": "P"}, {"code": "CM334", "description": "Applicant has no misdemeanor theft by check records in the last 5 years.", "result": "P"}, {"code": "CM335", "description": "Applicant has no felony traffic records in the last 10 years.", "result": "P"}, {"code": "CM337", "description": "Applicant has no felony violent crime records in the last 100 years.", "result": "P"}, {"code": "CM338", "description": "Applicant has no misdemeanor violent crime records in the last 5 years.", "result": "P"}, {"code": "CM339", "description": "Applicant has no felony weapons related in the last 100 years.", "result": "P"}, {"code": "CM340", "description": "Applicant has no misdemeanor weapons related in the last 5 years.", "result": "P"}, {"code": "RI400", "description": "Monthly rent is equal to or less than 36 % of Applicant's income.", "result": "--"}, {"code": "GI440", "description": "Monthly rent is equal to or less than 20 % of Guarantor's income.", "result": "P"}, {"code": "SX501", "description": "Applicant has no Name with DOB matches in the registered sex offender database.", "result": "P"}, {"code": "EV701", "description": "Applicant has less than 1 verified eviction records in the past 12 months.", "result": "P"}, {"code": "EV702", "description": "Applicant has less than 2 verified eviction initial filings in the past 12 months.", "result": "P"}, {"code": "CO807", "description": "Applicant has greater than 500 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "CO808", "description": "Applicant has greater than 1501 of outstanding rental collections debt in the past 24 months.", "result": "P"}, {"code": "SW849", "description": "Applicant has less than 1 late pays or NSF checks in the past 12 months in the First Advantage SkipWatch database.", "result": "P"}, {"code": "SW851", "description": "Applicant has less than 2 eviction notices in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SW852", "description": "Applicant has less than 1 eviction filed in the last 12 months in the First Advantage SkipWatch Database.", "result": "P"}, {"code": "SN901", "description": "Applicant has passed a Social Security Number fraud analysis.", "result": "F"}, {"code": "SN902", "description": "Social Security Number was provided?", "result": "F"}]</t>
+        </is>
+      </c>
+      <c r="AR19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AU19" t="n">
+        <v>2228</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="AX19" t="n">
+        <v>6189</v>
+      </c>
+      <c r="CY19" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP19" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DQ19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DS19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DT19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DU19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DV19" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DW19" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="DX19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DY19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="DZ19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EA19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EB19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EC19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ED19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EE19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EF19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EG19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EH19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EI19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EJ19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EK19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EL19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EM19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EN19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EO19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EP19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EQ19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ER19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ES19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="ET19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EU19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EV19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EW19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="EY19" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="EZ19" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="FA19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="FB19" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="FC19" t="inlineStr">
+        <is>
+          <t>32268854.htm</t>
+        </is>
+      </c>
+      <c r="FD19" t="inlineStr">
+        <is>
+          <t>06/10/2026 07:33:59 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TransUnion PDF</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07/09/2025</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>System User</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>22 North</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Ismael E Urbina</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>["Ismael Euceda", "Ismael Uceda"]</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>501 Horseshoe Dr, 1204 Leander TX 78641</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>512-203-8703</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Construction Leander, TX</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Exact SSN match</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Input (Current/Previous) Address is Commercial | Last name - input does not match file | Input SSN is not likely issued prior to June 2011.</t>
+        </is>
+      </c>
+      <c r="S20" t="b">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>3</v>
+      </c>
+      <c r="U20" t="n">
+        <v>592</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>ResidentScore 4.0</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>["Too many inquiries", "Not enough available credit", "Length of time revolving accounts have been established is too short", "Too few satisfactory accounts"]</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>{"revolving": {"count": 1, "high_credit": 0, "credit_limit": 500, "balance": 0, "past_due": 0, "payment": 0, "available": 100}, "installment": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "mortgage": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "open": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "closed_w_bal": {"count": null, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "total": {"count": 1, "high_credit": 0, "credit_limit": 500, "balance": 0, "past_due": 0, "payment": 0, "available": null}}</t>
+        </is>
+      </c>
+      <c r="AH20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>[{"creditor_name": "JPMCB CARD", "industry": "Banks", "loan_type": "Credit Card", "loan_terms": "Revolving", "account_type": "Individual account", "opened": "05/25", "verified": "06/25", "closed": null, "balance": 0, "past_due": 0, "credit_limit": 500, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}]</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>[{"date": "07/08/2025", "name": "ALLY FINANCI", "kind_of_business": "Finance or Personal"}, {"date": "07/08/2025", "name": "AUSTIN TELCO", "kind_of_business": "Credit Union and Finance Other Than Personal Companies"}, {"date": "07/08/2025", "name": "FIRST HELP F", "kind_of_business": "Finance or Personal"}, {"date": "07/08/2025", "name": "TOYOTA OF NO", "kind_of_business": "Automotive"}, {"date": "05/27/2025", "name": "RUNDRCKTYOTA", "kind_of_business": "Automotive"}, {"date": "05/23/2025", "name": "COVERT CHRYS", "kind_of_business": "Automotive"}, {"date": "04/28/2025", "name": "TOYOTA OF NO", "kind_of_business": "Automotive"}, {"date": "04/12/2025", "name": "SYNCB/LOWES", "kind_of_business": "Building Materials"}]</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>Too many inquiries</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>Not enough available credit</t>
+        </is>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>Length of time revolving accounts have been established is too short</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>Too few satisfactory accounts</t>
+        </is>
+      </c>
+      <c r="BC20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE20" t="n">
+        <v>500</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>100</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL20" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN20" t="n">
+        <v>500</v>
+      </c>
+      <c r="CO20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU20" t="n">
+        <v>500</v>
+      </c>
+      <c r="CW20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB20" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM20" t="n">
+        <v>8</v>
+      </c>
+      <c r="DN20" t="n">
+        <v>7</v>
+      </c>
+      <c r="DO20" t="inlineStr">
+        <is>
+          <t>07/08/2025</t>
+        </is>
+      </c>
+      <c r="FC20" t="inlineStr">
+        <is>
+          <t>CRER_2610_517309.pdf</t>
+        </is>
+      </c>
+      <c r="FD20" t="inlineStr">
+        <is>
+          <t>06/11/2026 08:51:30 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TransUnion PDF</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>System User</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>22 North</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Estheisy Y Villatoro pacheco</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Estheisy Villatoro; Estheisy Pacheco; Estheisy Villatoropacheco</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>3</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>3600 N Hills Dr, 115, Austin TX 78731</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>830 Fair Oaks Rd, 10, Houston TX 77023</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>501 Horseshoe Dr Leander, TX 78641</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>346-373-1954</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Exact match between SSN on input and on file.</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Current address mismatch - Input does not match file. | Input SSN likely not issued prior to June 2011</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="b">
+        <v>1</v>
+      </c>
+      <c r="T21" t="n">
+        <v>2</v>
+      </c>
+      <c r="U21" t="n">
+        <v>569</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>ResidentScore 4.0</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>["Too few revolving accounts", "Too many inquiries", "Not enough balance decreases on active non-mortgage accounts", "Balance of non-mortgage accounts is too high"]</t>
+        </is>
+      </c>
+      <c r="Y21" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>{"revolving": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "installment": {"count": 5, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "mortgage": {"count": 0, "high_credit": null, "credit_limit": null, "balance": null, "past_due": null, "payment": null, "available": null}, "open": {"count": 3, "high_credit": 3010, "credit_limit": 0, "balance": 263, "past_due": 0, "payment": 0, "available": 91}, "closed_w_bal": {"count": null, "high_credit": null, "credit_limit": null, "balance": 3797, "past_due": 3797, "payment": 0, "available": null}, "total": {"count": 8, "high_credit": 3010, "credit_limit": 0, "balance": 4060, "past_due": 3797, "payment": 0, "available": null}}</t>
+        </is>
+      </c>
+      <c r="AH21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>[{"creditor_name": "SHELL FCU", "industry": "Credit Union and Finance Other Than Personal Companies", "loan_type": null, "loan_terms": null, "account_type": null, "opened": "03/23", "verified": "01/26", "closed": "11/23", "balance": 1522, "past_due": 1522, "credit_limit": null, "payment_amount": null, "status": null, "remarks": null, "notes": null, "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "FEB/OPPLNS", "industry": "Finance or Personal", "loan_type": "Unsecured", "loan_terms": "Installment 009 Monthly", "account_type": "Individual account for sole use of consumer", "opened": "05/23", "verified": "01/26", "closed": "08/23", "balance": 1125, "past_due": 1125, "credit_limit": null, "payment_amount": null, "status": "Charged off as bad debt", "remarks": "Profit and loss writeoff", "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "OPORTUNPROG", "industry": "Finance or Personal", "loan_type": "Unsecured", "loan_terms": "Installment 012 Monthly", "account_type": "Individual account for sole use of consumer", "opened": "07/21", "verified": "05/22", "closed": "01/22", "balance": 1150, "past_due": 1150, "credit_limit": null, "payment_amount": null, "status": "Charged off as bad debt", "remarks": "Profit and loss writeoff", "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "CHIME-STRIDE", "industry": "Advertising", "loan_type": "Secured Credit Card", "loan_terms": "Open", "account_type": "Individual account for sole use of consumer", "opened": "11/25", "verified": "02/26", "closed": null, "balance": 263, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "CURRENT", "industry": "Advertising", "loan_type": "Unsecured", "loan_terms": "Installment 012 Monthly", "account_type": "Individual account for sole use of consumer", "opened": "12/25", "verified": null, "closed": null, "balance": 0, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Charged off as bad debt", "remarks": "Profit and loss writeoff", "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "FLEX", "industry": "Real Estate and Public Accommodations", "loan_type": "Rental Agreement", "loan_terms": "Open", "account_type": "Individual account for sole use of consumer", "opened": "09/25", "verified": "11/25", "closed": null, "balance": 0, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": null, "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "SHELL FCU", "industry": "Credit Union and Finance Other Than Personal Companies", "loan_type": "Unsecured", "loan_terms": "Installment 006 Monthly", "account_type": "Individual account for sole use of consumer", "opened": "08/22", "verified": "03/23", "closed": "03/23", "balance": 0, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": "Closed", "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}, {"creditor_name": "PREF LEASE", "industry": "Finance or Personal", "loan_type": "Rental Agreement", "loan_terms": "Installment 012 Monthly", "account_type": "Individual account for sole use of consumer", "opened": "05/21", "verified": "07/21", "closed": "07/21", "balance": 0, "past_due": 0, "credit_limit": null, "payment_amount": null, "status": "Paid or paying as agreed", "remarks": "Closed", "notes": "Automated account", "late_30": 0, "late_60": 0, "late_90": 0, "late_120_plus": 0}]</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>[{"collector_name": "CBE GROUP", "industry": "Collection services", "opened": "08/25", "verified": "02/26", "current_balance": 234, "original_balance": 234, "past_due": 234, "status": "Collection account", "remarks": "Placed for collection", "credit_grantor": "CHARTER COMMUNICATIONS"}, {"collector_name": "JEFFCAPSYS", "industry": "Collection services", "opened": "06/23", "verified": "02/26", "current_balance": 1150, "original_balance": 1150, "past_due": 1150, "status": "Collection account", "remarks": "Account information disputed by consumer", "credit_grantor": "OPORTUN INC"}, {"collector_name": "JEFFCAPSYS", "industry": "Collection services", "opened": "12/25", "verified": "02/26", "current_balance": 1129, "original_balance": 1129, "past_due": 1129, "status": "Collection account", "remarks": "Placed for collection", "credit_grantor": "T MOBILE"}, {"collector_name": "VANCEHUFFMAN", "industry": "Collection services", "opened": "03/25", "verified": "02/26", "current_balance": 1674, "original_balance": 1674, "past_due": 0, "status": "Collection account", "remarks": "Placed for collection", "credit_grantor": "CHECK N GO"}]</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>[{"date": "09/14/2024", "name": "CAPITAL ONE", "kind_of_business": "Banks"}, {"date": "09/02/2024", "name": "TITAN FACTORY DIRECT", "kind_of_business": "Miscellaneous"}]</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>Too few revolving accounts</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>Too many inquiries</t>
+        </is>
+      </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>Not enough balance decreases on active non-mortgage accounts</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>Balance of non-mortgage accounts is too high</t>
+        </is>
+      </c>
+      <c r="BC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
+      <c r="BJ21" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="inlineStr"/>
+      <c r="BP21" t="inlineStr"/>
+      <c r="BQ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR21" t="inlineStr"/>
+      <c r="BS21" t="inlineStr"/>
+      <c r="BT21" t="inlineStr"/>
+      <c r="BU21" t="inlineStr"/>
+      <c r="BV21" t="inlineStr"/>
+      <c r="BW21" t="inlineStr"/>
+      <c r="BX21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY21" t="n">
+        <v>3010</v>
+      </c>
+      <c r="BZ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA21" t="n">
+        <v>263</v>
+      </c>
+      <c r="CB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD21" t="n">
+        <v>91</v>
+      </c>
+      <c r="CE21" t="inlineStr"/>
+      <c r="CF21" t="inlineStr"/>
+      <c r="CG21" t="inlineStr"/>
+      <c r="CH21" t="n">
+        <v>3797</v>
+      </c>
+      <c r="CI21" t="n">
+        <v>3797</v>
+      </c>
+      <c r="CJ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK21" t="inlineStr"/>
+      <c r="CL21" t="n">
+        <v>8</v>
+      </c>
+      <c r="CM21" t="n">
+        <v>3010</v>
+      </c>
+      <c r="CN21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO21" t="n">
+        <v>4060</v>
+      </c>
+      <c r="CP21" t="n">
+        <v>3797</v>
+      </c>
+      <c r="CQ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR21" t="inlineStr"/>
+      <c r="CS21" t="n">
+        <v>4060</v>
+      </c>
+      <c r="CT21" t="n">
+        <v>3797</v>
+      </c>
+      <c r="CU21" t="inlineStr"/>
+      <c r="CV21" t="inlineStr"/>
+      <c r="CW21" t="n">
+        <v>1522</v>
+      </c>
+      <c r="CX21" t="n">
+        <v>1522</v>
+      </c>
+      <c r="CY21" t="n">
+        <v>3</v>
+      </c>
+      <c r="CZ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA21" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB21" t="n">
+        <v>3</v>
+      </c>
+      <c r="DC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH21" t="n">
+        <v>4187</v>
+      </c>
+      <c r="DI21" t="n">
+        <v>4187</v>
+      </c>
+      <c r="DJ21" t="n">
+        <v>2513</v>
+      </c>
+      <c r="DK21" t="n">
+        <v>1674</v>
+      </c>
+      <c r="DL21" t="n">
+        <v>4</v>
+      </c>
+      <c r="DM21" t="n">
+        <v>2</v>
+      </c>
+      <c r="DN21" t="n">
+        <v>2</v>
+      </c>
+      <c r="DO21" t="inlineStr">
+        <is>
+          <t>09/14/2024</t>
+        </is>
+      </c>
+      <c r="DP21" t="inlineStr"/>
+      <c r="DQ21" t="inlineStr"/>
+      <c r="DR21" t="inlineStr"/>
+      <c r="DS21" t="inlineStr"/>
+      <c r="DT21" t="inlineStr"/>
+      <c r="DU21" t="inlineStr"/>
+      <c r="DV21" t="inlineStr"/>
+      <c r="DW21" t="inlineStr"/>
+      <c r="DX21" t="inlineStr"/>
+      <c r="DY21" t="inlineStr"/>
+      <c r="DZ21" t="inlineStr"/>
+      <c r="EA21" t="inlineStr"/>
+      <c r="EB21" t="inlineStr"/>
+      <c r="EC21" t="inlineStr"/>
+      <c r="ED21" t="inlineStr"/>
+      <c r="EE21" t="inlineStr"/>
+      <c r="EF21" t="inlineStr"/>
+      <c r="EG21" t="inlineStr"/>
+      <c r="EH21" t="inlineStr"/>
+      <c r="EI21" t="inlineStr"/>
+      <c r="EJ21" t="inlineStr"/>
+      <c r="EK21" t="inlineStr"/>
+      <c r="EL21" t="inlineStr"/>
+      <c r="EM21" t="inlineStr"/>
+      <c r="EN21" t="inlineStr"/>
+      <c r="EO21" t="inlineStr"/>
+      <c r="EP21" t="inlineStr"/>
+      <c r="EQ21" t="inlineStr"/>
+      <c r="ER21" t="inlineStr"/>
+      <c r="ES21" t="inlineStr"/>
+      <c r="ET21" t="inlineStr"/>
+      <c r="EU21" t="inlineStr"/>
+      <c r="EV21" t="inlineStr"/>
+      <c r="EW21" t="inlineStr"/>
+      <c r="EX21" t="inlineStr"/>
+      <c r="EY21" t="inlineStr"/>
+      <c r="EZ21" t="inlineStr"/>
+      <c r="FA21" t="inlineStr"/>
+      <c r="FB21" t="inlineStr"/>
+      <c r="FC21" t="inlineStr">
+        <is>
+          <t>CRER_10685_533000.pdf</t>
+        </is>
+      </c>
+      <c r="FD21" t="inlineStr">
+        <is>
+          <t>06/11/2026 08:52:00 PM</t>
         </is>
       </c>
     </row>

</xml_diff>